<commit_message>
TICVAI r1.1: HLD/LLD, the Azure cost workbook and the decisions register rebuilt for the AI GPU node pool ($5,327.27 without HA, $8,295.04 with HA) and HOST-1 superseded in part (CHG-R11-001)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/hld-lld/TICVAI - Azure Cloud Specs & Cost.xlsx
+++ b/ticvai/handoff/hld-lld/TICVAI - Azure Cloud Specs & Cost.xlsx
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J72"/>
+  <dimension ref="A1:J74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -772,7 +772,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>AI pool: ticvai-ai, embedding model, reranker (CPU)</t>
+          <t>AI GPU pool: ticvai-ai, BGE-M3 and its reranker, Presidio and the Arabic NER (CHG-R11-001)</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -782,21 +782,21 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>D8s v5 (8 vCPU, 32 GB), Linux, autoscale 2-3. Two nodes are the least that carries the floors (real-time 2, interactive 1, 2 vCPU a pod) beside the embedding model and reranker (about 8 vCPU)</t>
+          <t>NV6ads A10 v5 (6 vCPU, 55 GB, 1/6 A10 with 4 GB), Linux, tainted, one node. Carries the floors (real-time 2, interactive 1, about 1 vCPU a pod) beside Presidio and, on the GPU, BGE-M3, its reranker and the Arabic NER. With the node down the scrubber is down and LLM calls are refused (503 scrubber-unavailable), never sent raw</t>
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>350</v>
+        <v>473.77</v>
       </c>
       <c r="I10" s="7">
         <f>G10*H10</f>
         <v/>
       </c>
       <c r="J10" s="7">
-        <f>3*H10</f>
+        <f>2*H10</f>
         <v/>
       </c>
     </row>
@@ -1772,238 +1772,168 @@
     <row r="42" ht="32" customHeight="1">
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>Node counts carry the replica floors of ADR-0061 (accepted 1 October): commerce 3, access 2, operations 2, workers 2, ticvai-ai real-time 2 (3 in a large cell), interactive 1, batch 0: 12 a cell, 13 in a large one. Pod sizes are assumptions until tools/bench.py measures them: about 1 vCPU for a .NET replica, 2 vCPU for an AI pod, about 8 vCPU for the embedding model and reranker together (AI design 4.3).</t>
+          <t>Node counts carry the replica floors of ADR-0061 (accepted 1 October): commerce 3, access 2, operations 2, workers 2, ticvai-ai real-time 2 (3 in a large cell), interactive 1, batch 0: 12 a cell, 13 in a large one. Pod sizes are assumptions until tools/bench.py measures them: about 1 vCPU for a .NET replica and about 1 vCPU for an AI pod, which mostly waits on the provider's streamed answer (AI design 4.3).</t>
         </is>
       </c>
     </row>
     <row r="43" ht="32" customHeight="1">
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>"When scaled up" doubles the autoscaled lines (workload and AI pools, Front Door traffic, bandwidth) for busy periods such as a holiday peak. A large on-sale runs in its own burst environment (ADR-0035, amended 3 September; deploy/c-flash-sale.yml), not priced here.</t>
+          <t>AI hosting (Chinmay, 4 October, CHG-R11-001): we host the embedding model (BGE-M3), its reranker, Presidio and the Arabic NER, together with the ticvai-ai pods, on one AI GPU node pool (NV6ads A10 v5, $473.77 a month a node; one node without HA, two with HA, one per zone); never an LLM, which stays with the providers (Core42 Compass, OpenAI UAE, BYOK). The 2 x D8s v5 AI CPU pool ($700) is gone: $8,047.50 became $8,295.04 with HA, $5,553.50 became $5,327.27 without. Defender for Containers is not re-priced for the GPU nodes' vCores (6 a node against the D8s v5's 8, so slightly lower). On AWS (me-central-1) the node is a g6.2xlarge-class instance (one L4, 8 vCPU), price and regional availability to confirm.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="32" customHeight="1">
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>Not included: Azure OpenAI tokens (billed per use), SMS, email and WhatsApp fees, payment provider fees, the e-invoicing provider (ADR-0062, proposed: the client names it), the DR module in UAE Central (bought per tenant), Apple and Google developer accounts, and venue hardware.</t>
+          <t>"When scaled up" doubles the autoscaled lines (workload and AI GPU pools, Front Door traffic, bandwidth) for busy periods such as a holiday peak. A large on-sale runs in its own burst environment (ADR-0035, amended 3 September; deploy/c-flash-sale.yml), not priced here.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="32" customHeight="1">
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>The venue edge node (one per venue, runs the gates and POS offline) is venue hardware, not Azure: recommended 8 cores, 32 GB RAM, 1 TB SSD, two units per venue for failover.</t>
+          <t>Not included: Azure OpenAI tokens (billed per use), SMS, email and WhatsApp fees, payment provider fees, the e-invoicing provider (ADR-0062, proposed: the client names it), the DR module in UAE Central (bought per tenant), Apple and Google developer accounts, and venue hardware.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="32" customHeight="1">
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>The event broker is the client's choice, due Monday 12 October (ADR-0057, proposed; docs/active/broker-decision-pack.md). We recommend RabbitMQ on CloudAMQP in UAE North: 3 nodes, $297-597 + $99 PrivateLink ($396-696), once 84codes confirms in writing that backups, settings and logs stay in UAE North. The sheet prices the fallback, RabbitMQ self-run on AKS (the Terraform default), because the plan is picked by the sprint-2 load test. Kafka alternatives: Event Hubs Standard with the Kafka endpoint $60-130 (10 topics per namespace); Premium 1 PU about $1,072; Confluent Cloud Enterprise about $1,280-1,640.</t>
+          <t>The venue edge node (one per venue, runs the gates and POS offline) is venue hardware, not Azure: recommended 8 cores, 32 GB RAM, 1 TB SSD, two units per venue for failover.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="32" customHeight="1">
       <c r="B47" s="14" t="inlineStr">
         <is>
-          <t>Front Door is a global service. It holds no personal data: it caches only public content (the on-sale waiting-room page, ADR-0066; public media such as the venue 3D models, ADR-0069) and decrypts at the edge nearest the user. Its WAF logs go to the UAE North Log Analytics workspace.</t>
+          <t>The event broker is the client's choice, due Monday 12 October (ADR-0057, proposed; docs/active/broker-decision-pack.md). We recommend RabbitMQ on CloudAMQP in UAE North: 3 nodes, $297-597 + $99 PrivateLink ($396-696), once 84codes confirms in writing that backups, settings and logs stay in UAE North. The sheet prices the fallback, RabbitMQ self-run on AKS (the Terraform default), because the plan is picked by the sprint-2 load test. Kafka alternatives: Event Hubs Standard with the Kafka endpoint $60-130 (10 topics per namespace); Premium 1 PU about $1,072; Confluent Cloud Enterprise about $1,280-1,640.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="32" customHeight="1">
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>Single zone for everything except PostgreSQL: a zone outage stops the cloud services until they are restored, and the database fails over to its standby. Venue gates and POS keep working on the venue edge node, offline.</t>
+          <t>Front Door is a global service. It holds no personal data: it caches only public content (the on-sale waiting-room page, ADR-0066; public media such as the venue 3D models, ADR-0069) and decrypts at the edge nearest the user. Its WAF logs go to the UAE North Log Analytics workspace.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="32" customHeight="1">
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>Not suitable for the cloud availability targets (ADR-0060, proposed: 99.95% for cloud commerce, 99.9% for the back office); use the high-availability sheet. Whether production may run this way is the client's answer to ADR-0060.</t>
+          <t>Single zone for everything except PostgreSQL: a zone outage stops the cloud services until they are restored, and the database fails over to its standby. Venue gates and POS keep working on the venue edge node, offline.</t>
         </is>
       </c>
     </row>
     <row r="50" ht="32" customHeight="1">
       <c r="B50" s="14" t="inlineStr">
         <is>
+          <t>Not suitable for the cloud availability targets (ADR-0060, proposed: 99.95% for cloud commerce, 99.9% for the back office); use the high-availability sheet. Whether production may run this way is the client's answer to ADR-0060.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="32" customHeight="1">
+      <c r="B51" s="14" t="inlineStr">
+        <is>
           <t>Recomputed 1 October 2026 (prices unchanged, those of 30 September): $4,531.50 became $5,553.50. PostgreSQL gains its zone-redundant standby, because production PostgreSQL is zone-redundant on every tier (ADR-0060, Chinmay, 1 October): +$320 compute, +$36 storage. A reporting replica of its own, because reporting never reads an operational replica (ADR-0016, the Terraform's enable_reporting_replica): +$196. A second AI node, because one node cannot hold the AI floors beside the embedding model and reranker (ADR-0061): +$350. The Private Link line the sheet lacked: +$50. Defender for the extra 8 vCores and the fourth PostgreSQL server: +$70.</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="3" t="inlineStr">
+    <row r="52" ht="32" customHeight="1">
+      <c r="B52" s="14" t="inlineStr">
+        <is>
+          <t>Recomputed 4 October 2026 (Chinmay, CHG-R11-001): the AI pool is one GPU node, NV6ads A10 v5 at $473.77, carrying the ticvai-ai pods, Presidio, the Arabic NER, BGE-M3 and its reranker, in place of the two D8s v5 AI nodes ($700): $5,553.50 became $5,327.27.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>Group</t>
         </is>
       </c>
-      <c r="C53" s="3" t="inlineStr">
+      <c r="C55" s="3" t="inlineStr">
         <is>
           <t>Azure service type</t>
         </is>
       </c>
-      <c r="D53" s="3" t="inlineStr">
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>Service description</t>
         </is>
       </c>
-      <c r="E53" s="3" t="inlineStr">
+      <c r="E55" s="3" t="inlineStr">
         <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="F53" s="3" t="inlineStr">
+      <c r="F55" s="3" t="inlineStr">
         <is>
           <t>Specs description</t>
         </is>
       </c>
-      <c r="G53" s="3" t="inlineStr">
+      <c r="G55" s="3" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="H53" s="3" t="inlineStr">
+      <c r="H55" s="3" t="inlineStr">
         <is>
           <t>Unit price (USD / month)</t>
         </is>
       </c>
-      <c r="I53" s="3" t="inlineStr">
+      <c r="I55" s="3" t="inlineStr">
         <is>
           <t>Estimated monthly cost (USD)</t>
         </is>
       </c>
-      <c r="J53" s="3" t="inlineStr">
+      <c r="J55" s="3" t="inlineStr">
         <is>
           <t>When solution is scaled up (USD)</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="4" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>Pre-production</t>
         </is>
       </c>
-      <c r="B54" s="5" t="inlineStr">
+      <c r="B56" s="5" t="inlineStr">
         <is>
           <t>Compute (AKS)</t>
         </is>
       </c>
-      <c r="C54" s="5" t="inlineStr">
+      <c r="C56" s="5" t="inlineStr">
         <is>
           <t>Azure Kubernetes Service</t>
         </is>
       </c>
-      <c r="D54" s="5" t="inlineStr">
+      <c r="D56" s="5" t="inlineStr">
         <is>
           <t>Control plane</t>
         </is>
       </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>UAE North</t>
-        </is>
-      </c>
-      <c r="F54" s="5" t="inlineStr">
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>UAE North</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
         <is>
           <t>Free tier</t>
         </is>
       </c>
-      <c r="G54" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H54" s="6" t="n">
+      <c r="G56" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H56" s="6" t="n">
         <v>0</v>
-      </c>
-      <c r="I54" s="7">
-        <f>G54*H54</f>
-        <v/>
-      </c>
-      <c r="J54" s="7">
-        <f>I54</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="n"/>
-      <c r="B55" s="5" t="inlineStr">
-        <is>
-          <t>Compute (AKS)</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>Virtual Machines (AKS nodes)</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>System and workload nodes, all five deployables</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>UAE North</t>
-        </is>
-      </c>
-      <c r="F55" s="5" t="inlineStr">
-        <is>
-          <t>D8s v5 (8 vCPU, 32 GB) x2 + D4s v5 x1, Linux. One replica per unit: the ADR-0061 floors are for production cells</t>
-        </is>
-      </c>
-      <c r="G55" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H55" s="6" t="n">
-        <v>875</v>
-      </c>
-      <c r="I55" s="7">
-        <f>G55*H55</f>
-        <v/>
-      </c>
-      <c r="J55" s="7">
-        <f>I55</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="n"/>
-      <c r="B56" s="5" t="inlineStr">
-        <is>
-          <t>Vector store</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>Virtual Machines (AKS nodes)</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>Qdrant, single node</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>UAE North</t>
-        </is>
-      </c>
-      <c r="F56" s="5" t="inlineStr">
-        <is>
-          <t>E2s v5 (2 vCPU, 16 GB) + P10 128 GB</t>
-        </is>
-      </c>
-      <c r="G56" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H56" s="6" t="n">
-        <v>132</v>
       </c>
       <c r="I56" s="7">
         <f>G56*H56</f>
@@ -2018,7 +1948,7 @@
       <c r="A57" s="8" t="n"/>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>Event broker</t>
+          <t>Compute (AKS)</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
@@ -2028,7 +1958,7 @@
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>RabbitMQ, single node, whichever broker production uses</t>
+          <t>System and workload nodes, all five deployables</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -2038,14 +1968,14 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>D2s v5 (2 vCPU, 8 GB). With Kafka in production, add an Event Hubs Standard namespace (about $30)</t>
+          <t>D8s v5 (8 vCPU, 32 GB) x2 + D4s v5 x1, Linux. One replica per unit: the ADR-0061 floors are for production cells</t>
         </is>
       </c>
       <c r="G57" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H57" s="6" t="n">
-        <v>88</v>
+        <v>875</v>
       </c>
       <c r="I57" s="7">
         <f>G57*H57</f>
@@ -2060,17 +1990,17 @@
       <c r="A58" s="8" t="n"/>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>Event broker</t>
+          <t>Vector store</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Managed Disks</t>
+          <t>Virtual Machines (AKS nodes)</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Broker storage</t>
+          <t>Qdrant, single node</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -2080,14 +2010,14 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>Premium SSD P10 128 GB</t>
+          <t>E2s v5 (2 vCPU, 16 GB) + P10 128 GB</t>
         </is>
       </c>
       <c r="G58" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H58" s="6" t="n">
-        <v>21.5</v>
+        <v>132</v>
       </c>
       <c r="I58" s="7">
         <f>G58*H58</f>
@@ -2102,17 +2032,17 @@
       <c r="A59" s="8" t="n"/>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Database</t>
+          <t>Event broker</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Azure Database for PostgreSQL</t>
+          <t>Virtual Machines (AKS nodes)</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>Control DB + test tenant DBs + AI log DB</t>
+          <t>RabbitMQ, single node, whichever broker production uses</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -2122,14 +2052,14 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>Flexible Server 16, General Purpose D2ds v5 + 256 GB, no standby (database_high_availability = false: pre-production only), no replicas</t>
+          <t>D2s v5 (2 vCPU, 8 GB). With Kafka in production, add an Event Hubs Standard namespace (about $30)</t>
         </is>
       </c>
       <c r="G59" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H59" s="6" t="n">
-        <v>196</v>
+        <v>88</v>
       </c>
       <c r="I59" s="7">
         <f>G59*H59</f>
@@ -2144,17 +2074,17 @@
       <c r="A60" s="8" t="n"/>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>Cache</t>
+          <t>Event broker</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Azure Managed Redis</t>
+          <t>Managed Disks</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>Test cache</t>
+          <t>Broker storage</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -2164,14 +2094,14 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>Balanced B1 (1 GB), one node (B0, about $53, if enough)</t>
+          <t>Premium SSD P10 128 GB</t>
         </is>
       </c>
       <c r="G60" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H60" s="6" t="n">
-        <v>133</v>
+        <v>21.5</v>
       </c>
       <c r="I60" s="7">
         <f>G60*H60</f>
@@ -2186,17 +2116,17 @@
       <c r="A61" s="8" t="n"/>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Storage</t>
+          <t>Database</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Storage account (Blob, LRS)</t>
+          <t>Azure Database for PostgreSQL</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Test media and snapshots</t>
+          <t>Control DB + test tenant DBs + AI log DB</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -2206,14 +2136,14 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>Hot tier, 500 GB</t>
+          <t>Flexible Server 16, General Purpose D2ds v5 + 256 GB, no standby (database_high_availability = false: pre-production only), no replicas</t>
         </is>
       </c>
       <c r="G61" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H61" s="6" t="n">
-        <v>15</v>
+        <v>196</v>
       </c>
       <c r="I61" s="7">
         <f>G61*H61</f>
@@ -2228,17 +2158,17 @@
       <c r="A62" s="8" t="n"/>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Cache</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Key Vault</t>
+          <t>Azure Managed Redis</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>Test secrets</t>
+          <t>Test cache</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -2248,14 +2178,14 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Balanced B1 (1 GB), one node (B0, about $53, if enough)</t>
         </is>
       </c>
       <c r="G62" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H62" s="6" t="n">
-        <v>5</v>
+        <v>133</v>
       </c>
       <c r="I62" s="7">
         <f>G62*H62</f>
@@ -2270,17 +2200,17 @@
       <c r="A63" s="8" t="n"/>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Network</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Front Door, NAT, Bastion, Registry</t>
+          <t>Storage account (Blob, LRS)</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>Shared with production</t>
+          <t>Test media and snapshots</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -2290,14 +2220,14 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>Separate routes and WAF policy</t>
+          <t>Hot tier, 500 GB</t>
         </is>
       </c>
       <c r="G63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H63" s="6" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="I63" s="7">
         <f>G63*H63</f>
@@ -2309,20 +2239,20 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="9" t="n"/>
+      <c r="A64" s="8" t="n"/>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Azure Monitor / Log Analytics</t>
+          <t>Key Vault</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>Logs and metrics</t>
+          <t>Test secrets</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -2332,14 +2262,14 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>About 20 GB ingested a month</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="G64" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H64" s="6" t="n">
-        <v>70</v>
+        <v>5</v>
       </c>
       <c r="I64" s="7">
         <f>G64*H64</f>
@@ -2351,97 +2281,183 @@
       </c>
     </row>
     <row r="65">
-      <c r="F65" s="10" t="inlineStr">
-        <is>
-          <t>USD - Total cost per month</t>
-        </is>
-      </c>
-      <c r="I65" s="11">
-        <f>SUM(I54:I64)</f>
-        <v/>
-      </c>
-      <c r="J65" s="12">
-        <f>SUM(J54:J64)</f>
+      <c r="A65" s="8" t="n"/>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>Network</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>Front Door, NAT, Bastion, Registry</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Shared with production</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>UAE North</t>
+        </is>
+      </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>Separate routes and WAF policy</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H65" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I65" s="7">
+        <f>G65*H65</f>
+        <v/>
+      </c>
+      <c r="J65" s="7">
+        <f>I65</f>
         <v/>
       </c>
     </row>
     <row r="66">
-      <c r="F66" s="10" t="inlineStr">
-        <is>
-          <t>AED - Total cost per month</t>
-        </is>
-      </c>
-      <c r="I66" s="11">
-        <f>I65*$C$3</f>
-        <v/>
-      </c>
-      <c r="J66" s="12">
-        <f>J65*$C$3</f>
+      <c r="A66" s="9" t="n"/>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>Azure Monitor / Log Analytics</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Logs and metrics</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>UAE North</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>About 20 GB ingested a month</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H66" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="I66" s="7">
+        <f>G66*H66</f>
+        <v/>
+      </c>
+      <c r="J66" s="7">
+        <f>I66</f>
         <v/>
       </c>
     </row>
     <row r="67">
       <c r="F67" s="10" t="inlineStr">
         <is>
-          <t>AED - Total cost per year</t>
+          <t>USD - Total cost per month</t>
         </is>
       </c>
       <c r="I67" s="11">
-        <f>I66*12</f>
+        <f>SUM(I56:I66)</f>
+        <v/>
+      </c>
+      <c r="J67" s="12">
+        <f>SUM(J56:J66)</f>
         <v/>
       </c>
     </row>
     <row r="68">
       <c r="F68" s="10" t="inlineStr">
         <is>
+          <t>AED - Total cost per month</t>
+        </is>
+      </c>
+      <c r="I68" s="11">
+        <f>I67*$C$3</f>
+        <v/>
+      </c>
+      <c r="J68" s="12">
+        <f>J67*$C$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="F69" s="10" t="inlineStr">
+        <is>
+          <t>AED - Total cost per year</t>
+        </is>
+      </c>
+      <c r="I69" s="11">
+        <f>I68*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="F70" s="10" t="inlineStr">
+        <is>
           <t>AED - Total price per year with margin</t>
         </is>
       </c>
-      <c r="I68" s="11">
-        <f>I67*(1+$C$4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70">
-      <c r="B70" s="13" t="inlineStr">
+      <c r="I70" s="11">
+        <f>I69*(1+$C$4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="13" t="inlineStr">
         <is>
           <t>Notes - Pre-production</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="32" customHeight="1">
-      <c r="B71" s="14" t="inlineStr">
+    <row r="73" ht="32" customHeight="1">
+      <c r="B73" s="14" t="inlineStr">
         <is>
           <t>One pre-production environment for acceptance testing and client demos; development runs locally on docker-compose (deploy/*.yml) and on this cluster.</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="32" customHeight="1">
-      <c r="B72" s="14" t="inlineStr">
+    <row r="74" ht="32" customHeight="1">
+      <c r="B74" s="14" t="inlineStr">
         <is>
           <t>Zero-priced lines are covered by production.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="B44:I44"/>
-    <mergeCell ref="B48:I48"/>
-    <mergeCell ref="A7:A31"/>
-    <mergeCell ref="B39:I39"/>
-    <mergeCell ref="B38:I38"/>
+  <mergeCells count="19">
     <mergeCell ref="B47:I47"/>
     <mergeCell ref="B46:I46"/>
+    <mergeCell ref="B43:I43"/>
+    <mergeCell ref="B52:I52"/>
+    <mergeCell ref="A56:A66"/>
+    <mergeCell ref="B48:I48"/>
+    <mergeCell ref="B39:I39"/>
     <mergeCell ref="B42:I42"/>
-    <mergeCell ref="B72:I72"/>
-    <mergeCell ref="A54:A64"/>
+    <mergeCell ref="B73:I73"/>
+    <mergeCell ref="B44:I44"/>
+    <mergeCell ref="B38:I38"/>
+    <mergeCell ref="B49:I49"/>
+    <mergeCell ref="B40:I40"/>
+    <mergeCell ref="B74:I74"/>
+    <mergeCell ref="A7:A31"/>
+    <mergeCell ref="B51:I51"/>
     <mergeCell ref="B45:I45"/>
-    <mergeCell ref="B43:I43"/>
     <mergeCell ref="B41:I41"/>
-    <mergeCell ref="B71:I71"/>
-    <mergeCell ref="B49:I49"/>
     <mergeCell ref="B50:I50"/>
-    <mergeCell ref="B40:I40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2453,7 +2469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J72"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2701,7 +2717,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>AI pool: ticvai-ai, embedding model, reranker (CPU)</t>
+          <t>AI GPU pool: ticvai-ai, BGE-M3 and its reranker, Presidio and the Arabic NER (CHG-R11-001)</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -2711,14 +2727,14 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>D8s v5 (8 vCPU, 32 GB), Linux, autoscale 2-4, tainted. Carries the floors: real-time 2, interactive 1, batch 0 (2 vCPU a pod) beside the embedding model and reranker (about 8 vCPU). A large cell's third real-time replica takes a third node</t>
+          <t>NV6ads A10 v5 (6 vCPU, 55 GB, 1/6 A10 with 4 GB), Linux, tainted, one node per zone. Carries the floors: real-time 2, interactive 1, batch 0 (about 1 vCPU a pod), Presidio on the CPU, and on the GPU at fp16 BGE-M3 (about 1.1 GB), its reranker (about 1.1 GB) and the Arabic NER (about 0.3 GB); a large cell's third real-time replica fits. No AI CPU pool and no Presidio pool. Sizing to confirm by the Sprint 2 benchmark; step up to NV12ads A10 v5 ($947.54) on CPU saturation or GPU memory pressure. AWS me-central-1: a g6.2xlarge-class node, price to confirm</t>
         </is>
       </c>
       <c r="G10" s="5" t="n">
         <v>2</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>350</v>
+        <v>473.77</v>
       </c>
       <c r="I10" s="7">
         <f>G10*H10</f>
@@ -3743,189 +3759,154 @@
     <row r="43" ht="32" customHeight="1">
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>Node counts carry the replica floors of ADR-0061 (accepted 1 October): commerce 3, access 2, operations 2, workers 2, ticvai-ai real-time 2 (3 in a large cell), interactive 1, batch 0: 12 a cell, 13 in a large one. Pod sizes are assumptions until tools/bench.py measures them: about 1 vCPU for a .NET replica, 2 vCPU for an AI pod, about 8 vCPU for the embedding model and reranker together (AI design 4.3).</t>
+          <t>Node counts carry the replica floors of ADR-0061 (accepted 1 October): commerce 3, access 2, operations 2, workers 2, ticvai-ai real-time 2 (3 in a large cell), interactive 1, batch 0: 12 a cell, 13 in a large one. Pod sizes are assumptions until tools/bench.py measures them: about 1 vCPU for a .NET replica and about 1 vCPU for an AI pod, which mostly waits on the provider's streamed answer (AI design 4.3).</t>
         </is>
       </c>
     </row>
     <row r="44" ht="32" customHeight="1">
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>"When scaled up" doubles the autoscaled lines (workload and AI pools, Front Door traffic, bandwidth) for busy periods such as a holiday peak. A large on-sale runs in its own burst environment (ADR-0035, amended 3 September; deploy/c-flash-sale.yml), not priced here.</t>
+          <t>AI hosting (Chinmay, 4 October, CHG-R11-001): we host the embedding model (BGE-M3), its reranker, Presidio and the Arabic NER, together with the ticvai-ai pods, on one AI GPU node pool (NV6ads A10 v5, $473.77 a month a node; one node without HA, two with HA, one per zone); never an LLM, which stays with the providers (Core42 Compass, OpenAI UAE, BYOK). The 2 x D8s v5 AI CPU pool ($700) is gone: $8,047.50 became $8,295.04 with HA, $5,553.50 became $5,327.27 without. Defender for Containers is not re-priced for the GPU nodes' vCores (6 a node against the D8s v5's 8, so slightly lower). On AWS (me-central-1) the node is a g6.2xlarge-class instance (one L4, 8 vCPU), price and regional availability to confirm.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="32" customHeight="1">
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>Not included: Azure OpenAI tokens (billed per use), SMS, email and WhatsApp fees, payment provider fees, the e-invoicing provider (ADR-0062, proposed: the client names it), the DR module in UAE Central (bought per tenant), Apple and Google developer accounts, and venue hardware.</t>
+          <t>"When scaled up" doubles the autoscaled lines (workload and AI GPU pools, Front Door traffic, bandwidth) for busy periods such as a holiday peak. A large on-sale runs in its own burst environment (ADR-0035, amended 3 September; deploy/c-flash-sale.yml), not priced here.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="32" customHeight="1">
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>The venue edge node (one per venue, runs the gates and POS offline) is venue hardware, not Azure: recommended 8 cores, 32 GB RAM, 1 TB SSD, two units per venue for failover.</t>
+          <t>Not included: Azure OpenAI tokens (billed per use), SMS, email and WhatsApp fees, payment provider fees, the e-invoicing provider (ADR-0062, proposed: the client names it), the DR module in UAE Central (bought per tenant), Apple and Google developer accounts, and venue hardware.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="32" customHeight="1">
       <c r="B47" s="14" t="inlineStr">
         <is>
-          <t>The event broker is the client's choice, due Monday 12 October (ADR-0057, proposed; docs/active/broker-decision-pack.md). We recommend RabbitMQ on CloudAMQP in UAE North: 3 nodes, $297-597 + $99 PrivateLink ($396-696), once 84codes confirms in writing that backups, settings and logs stay in UAE North. The sheet prices the fallback, RabbitMQ self-run on AKS (the Terraform default), because the plan is picked by the sprint-2 load test. Kafka alternatives: Event Hubs Standard with the Kafka endpoint $60-130 (10 topics per namespace); Premium 1 PU about $1,072; Confluent Cloud Enterprise about $1,280-1,640.</t>
+          <t>The venue edge node (one per venue, runs the gates and POS offline) is venue hardware, not Azure: recommended 8 cores, 32 GB RAM, 1 TB SSD, two units per venue for failover.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="32" customHeight="1">
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>Front Door is a global service. It holds no personal data: it caches only public content (the on-sale waiting-room page, ADR-0066; public media such as the venue 3D models, ADR-0069) and decrypts at the edge nearest the user. Its WAF logs go to the UAE North Log Analytics workspace.</t>
+          <t>The event broker is the client's choice, due Monday 12 October (ADR-0057, proposed; docs/active/broker-decision-pack.md). We recommend RabbitMQ on CloudAMQP in UAE North: 3 nodes, $297-597 + $99 PrivateLink ($396-696), once 84codes confirms in writing that backups, settings and logs stay in UAE North. The sheet prices the fallback, RabbitMQ self-run on AKS (the Terraform default), because the plan is picked by the sprint-2 load test. Kafka alternatives: Event Hubs Standard with the Kafka endpoint $60-130 (10 topics per namespace); Premium 1 PU about $1,072; Confluent Cloud Enterprise about $1,280-1,640.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="32" customHeight="1">
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>Zones 1-3 in UAE North: PostgreSQL zone-redundant standby (on every production tier, ADR-0060), Qdrant and broker three-node clusters, AKS node pools across zones, Azure Managed Redis with high availability (zone-redundant). This is the shape of a shared cell and of a dedicated one.</t>
+          <t>Front Door is a global service. It holds no personal data: it caches only public content (the on-sale waiting-room page, ADR-0066; public media such as the venue 3D models, ADR-0069) and decrypts at the edge nearest the user. Its WAF logs go to the UAE North Log Analytics workspace.</t>
         </is>
       </c>
     </row>
     <row r="50" ht="32" customHeight="1">
       <c r="B50" s="14" t="inlineStr">
         <is>
+          <t>Zones 1-3 in UAE North: PostgreSQL zone-redundant standby (on every production tier, ADR-0060), Qdrant and broker three-node clusters, AKS node pools across zones, Azure Managed Redis with high availability (zone-redundant). This is the shape of a shared cell and of a dedicated one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="32" customHeight="1">
+      <c r="B51" s="14" t="inlineStr">
+        <is>
           <t>Availability targets per tier (ADR-0060, proposed, with the client): 99.99% for venue operations (gate, POS, KDS) measured locally; 99.95% for commerce in the cloud; 99.9% for back office and operations; 99.5% for AI and engagement. Only an active-active, two-region design reaches 99.99% for the whole cloud path.</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="3" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B54" s="3" t="inlineStr">
         <is>
           <t>Group</t>
         </is>
       </c>
-      <c r="C53" s="3" t="inlineStr">
+      <c r="C54" s="3" t="inlineStr">
         <is>
           <t>Azure service type</t>
         </is>
       </c>
-      <c r="D53" s="3" t="inlineStr">
+      <c r="D54" s="3" t="inlineStr">
         <is>
           <t>Service description</t>
         </is>
       </c>
-      <c r="E53" s="3" t="inlineStr">
+      <c r="E54" s="3" t="inlineStr">
         <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="F53" s="3" t="inlineStr">
+      <c r="F54" s="3" t="inlineStr">
         <is>
           <t>Specs description</t>
         </is>
       </c>
-      <c r="G53" s="3" t="inlineStr">
+      <c r="G54" s="3" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="H53" s="3" t="inlineStr">
+      <c r="H54" s="3" t="inlineStr">
         <is>
           <t>Unit price (USD / month)</t>
         </is>
       </c>
-      <c r="I53" s="3" t="inlineStr">
+      <c r="I54" s="3" t="inlineStr">
         <is>
           <t>Estimated monthly cost (USD)</t>
         </is>
       </c>
-      <c r="J53" s="3" t="inlineStr">
+      <c r="J54" s="3" t="inlineStr">
         <is>
           <t>When solution is scaled up (USD)</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="4" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
         <is>
           <t>Pre-production</t>
         </is>
       </c>
-      <c r="B54" s="5" t="inlineStr">
+      <c r="B55" s="5" t="inlineStr">
         <is>
           <t>Compute (AKS)</t>
         </is>
       </c>
-      <c r="C54" s="5" t="inlineStr">
+      <c r="C55" s="5" t="inlineStr">
         <is>
           <t>Azure Kubernetes Service</t>
         </is>
       </c>
-      <c r="D54" s="5" t="inlineStr">
+      <c r="D55" s="5" t="inlineStr">
         <is>
           <t>Control plane</t>
         </is>
       </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>UAE North</t>
-        </is>
-      </c>
-      <c r="F54" s="5" t="inlineStr">
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>UAE North</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
         <is>
           <t>Free tier</t>
         </is>
       </c>
-      <c r="G54" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H54" s="6" t="n">
+      <c r="G55" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H55" s="6" t="n">
         <v>0</v>
-      </c>
-      <c r="I54" s="7">
-        <f>G54*H54</f>
-        <v/>
-      </c>
-      <c r="J54" s="7">
-        <f>I54</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="n"/>
-      <c r="B55" s="5" t="inlineStr">
-        <is>
-          <t>Compute (AKS)</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>Virtual Machines (AKS nodes)</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>System and workload nodes, all five deployables</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>UAE North</t>
-        </is>
-      </c>
-      <c r="F55" s="5" t="inlineStr">
-        <is>
-          <t>D8s v5 (8 vCPU, 32 GB) x2 + D4s v5 x1, Linux. One replica per unit: the ADR-0061 floors are for production cells</t>
-        </is>
-      </c>
-      <c r="G55" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H55" s="6" t="n">
-        <v>875</v>
       </c>
       <c r="I55" s="7">
         <f>G55*H55</f>
@@ -3940,7 +3921,7 @@
       <c r="A56" s="8" t="n"/>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Vector store</t>
+          <t>Compute (AKS)</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
@@ -3950,7 +3931,7 @@
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Qdrant, single node</t>
+          <t>System and workload nodes, all five deployables</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -3960,14 +3941,14 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>E2s v5 (2 vCPU, 16 GB) + P10 128 GB</t>
+          <t>D8s v5 (8 vCPU, 32 GB) x2 + D4s v5 x1, Linux. One replica per unit: the ADR-0061 floors are for production cells</t>
         </is>
       </c>
       <c r="G56" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H56" s="6" t="n">
-        <v>132</v>
+        <v>875</v>
       </c>
       <c r="I56" s="7">
         <f>G56*H56</f>
@@ -3982,7 +3963,7 @@
       <c r="A57" s="8" t="n"/>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>Event broker</t>
+          <t>Vector store</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
@@ -3992,7 +3973,7 @@
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>RabbitMQ, single node, whichever broker production uses</t>
+          <t>Qdrant, single node</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -4002,14 +3983,14 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>D2s v5 (2 vCPU, 8 GB). With Kafka in production, add an Event Hubs Standard namespace (about $30)</t>
+          <t>E2s v5 (2 vCPU, 16 GB) + P10 128 GB</t>
         </is>
       </c>
       <c r="G57" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H57" s="6" t="n">
-        <v>88</v>
+        <v>132</v>
       </c>
       <c r="I57" s="7">
         <f>G57*H57</f>
@@ -4029,12 +4010,12 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Managed Disks</t>
+          <t>Virtual Machines (AKS nodes)</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Broker storage</t>
+          <t>RabbitMQ, single node, whichever broker production uses</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -4044,14 +4025,14 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>Premium SSD P10 128 GB</t>
+          <t>D2s v5 (2 vCPU, 8 GB). With Kafka in production, add an Event Hubs Standard namespace (about $30)</t>
         </is>
       </c>
       <c r="G58" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H58" s="6" t="n">
-        <v>21.5</v>
+        <v>88</v>
       </c>
       <c r="I58" s="7">
         <f>G58*H58</f>
@@ -4066,17 +4047,17 @@
       <c r="A59" s="8" t="n"/>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Database</t>
+          <t>Event broker</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Azure Database for PostgreSQL</t>
+          <t>Managed Disks</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>Control DB + test tenant DBs + AI log DB</t>
+          <t>Broker storage</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -4086,14 +4067,14 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>Flexible Server 16, General Purpose D2ds v5 + 256 GB, no standby (database_high_availability = false: pre-production only), no replicas</t>
+          <t>Premium SSD P10 128 GB</t>
         </is>
       </c>
       <c r="G59" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H59" s="6" t="n">
-        <v>196</v>
+        <v>21.5</v>
       </c>
       <c r="I59" s="7">
         <f>G59*H59</f>
@@ -4108,17 +4089,17 @@
       <c r="A60" s="8" t="n"/>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>Cache</t>
+          <t>Database</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Azure Managed Redis</t>
+          <t>Azure Database for PostgreSQL</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>Test cache</t>
+          <t>Control DB + test tenant DBs + AI log DB</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -4128,14 +4109,14 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>Balanced B1 (1 GB), one node (B0, about $53, if enough)</t>
+          <t>Flexible Server 16, General Purpose D2ds v5 + 256 GB, no standby (database_high_availability = false: pre-production only), no replicas</t>
         </is>
       </c>
       <c r="G60" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H60" s="6" t="n">
-        <v>133</v>
+        <v>196</v>
       </c>
       <c r="I60" s="7">
         <f>G60*H60</f>
@@ -4150,17 +4131,17 @@
       <c r="A61" s="8" t="n"/>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Storage</t>
+          <t>Cache</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Storage account (Blob, LRS)</t>
+          <t>Azure Managed Redis</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Test media and snapshots</t>
+          <t>Test cache</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -4170,14 +4151,14 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>Hot tier, 500 GB</t>
+          <t>Balanced B1 (1 GB), one node (B0, about $53, if enough)</t>
         </is>
       </c>
       <c r="G61" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H61" s="6" t="n">
-        <v>15</v>
+        <v>133</v>
       </c>
       <c r="I61" s="7">
         <f>G61*H61</f>
@@ -4192,17 +4173,17 @@
       <c r="A62" s="8" t="n"/>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Key Vault</t>
+          <t>Storage account (Blob, LRS)</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>Test secrets</t>
+          <t>Test media and snapshots</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -4212,14 +4193,14 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Hot tier, 500 GB</t>
         </is>
       </c>
       <c r="G62" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H62" s="6" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="I62" s="7">
         <f>G62*H62</f>
@@ -4234,17 +4215,17 @@
       <c r="A63" s="8" t="n"/>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Network</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Front Door, NAT, Bastion, Registry</t>
+          <t>Key Vault</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>Shared with production</t>
+          <t>Test secrets</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -4254,14 +4235,14 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>Separate routes and WAF policy</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="G63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H63" s="6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I63" s="7">
         <f>G63*H63</f>
@@ -4273,20 +4254,20 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="9" t="n"/>
+      <c r="A64" s="8" t="n"/>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Network</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Azure Monitor / Log Analytics</t>
+          <t>Front Door, NAT, Bastion, Registry</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>Logs and metrics</t>
+          <t>Shared with production</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -4296,14 +4277,14 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>About 20 GB ingested a month</t>
+          <t>Separate routes and WAF policy</t>
         </is>
       </c>
       <c r="G64" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H64" s="6" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="I64" s="7">
         <f>G64*H64</f>
@@ -4315,93 +4296,136 @@
       </c>
     </row>
     <row r="65">
-      <c r="F65" s="10" t="inlineStr">
-        <is>
-          <t>USD - Total cost per month</t>
-        </is>
-      </c>
-      <c r="I65" s="11">
-        <f>SUM(I54:I64)</f>
-        <v/>
-      </c>
-      <c r="J65" s="12">
-        <f>SUM(J54:J64)</f>
+      <c r="A65" s="9" t="n"/>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>Azure Monitor / Log Analytics</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Logs and metrics</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>UAE North</t>
+        </is>
+      </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>About 20 GB ingested a month</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H65" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="I65" s="7">
+        <f>G65*H65</f>
+        <v/>
+      </c>
+      <c r="J65" s="7">
+        <f>I65</f>
         <v/>
       </c>
     </row>
     <row r="66">
       <c r="F66" s="10" t="inlineStr">
         <is>
-          <t>AED - Total cost per month</t>
+          <t>USD - Total cost per month</t>
         </is>
       </c>
       <c r="I66" s="11">
-        <f>I65*$C$3</f>
+        <f>SUM(I55:I65)</f>
         <v/>
       </c>
       <c r="J66" s="12">
-        <f>J65*$C$3</f>
+        <f>SUM(J55:J65)</f>
         <v/>
       </c>
     </row>
     <row r="67">
       <c r="F67" s="10" t="inlineStr">
         <is>
-          <t>AED - Total cost per year</t>
+          <t>AED - Total cost per month</t>
         </is>
       </c>
       <c r="I67" s="11">
-        <f>I66*12</f>
+        <f>I66*$C$3</f>
+        <v/>
+      </c>
+      <c r="J67" s="12">
+        <f>J66*$C$3</f>
         <v/>
       </c>
     </row>
     <row r="68">
       <c r="F68" s="10" t="inlineStr">
         <is>
+          <t>AED - Total cost per year</t>
+        </is>
+      </c>
+      <c r="I68" s="11">
+        <f>I67*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="F69" s="10" t="inlineStr">
+        <is>
           <t>AED - Total price per year with margin</t>
         </is>
       </c>
-      <c r="I68" s="11">
-        <f>I67*(1+$C$4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70">
-      <c r="B70" s="13" t="inlineStr">
+      <c r="I69" s="11">
+        <f>I68*(1+$C$4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="13" t="inlineStr">
         <is>
           <t>Notes - Pre-production</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="32" customHeight="1">
-      <c r="B71" s="14" t="inlineStr">
-        <is>
-          <t>One pre-production environment for acceptance testing and client demos; development runs locally on docker-compose (deploy/*.yml) and on this cluster.</t>
         </is>
       </c>
     </row>
     <row r="72" ht="32" customHeight="1">
       <c r="B72" s="14" t="inlineStr">
         <is>
+          <t>One pre-production environment for acceptance testing and client demos; development runs locally on docker-compose (deploy/*.yml) and on this cluster.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="32" customHeight="1">
+      <c r="B73" s="14" t="inlineStr">
+        <is>
           <t>Zero-priced lines are covered by production.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="17">
+    <mergeCell ref="B73:I73"/>
     <mergeCell ref="B44:I44"/>
     <mergeCell ref="B48:I48"/>
     <mergeCell ref="B45:I45"/>
     <mergeCell ref="B39:I39"/>
+    <mergeCell ref="A55:A65"/>
     <mergeCell ref="B47:I47"/>
+    <mergeCell ref="B51:I51"/>
     <mergeCell ref="B46:I46"/>
     <mergeCell ref="B42:I42"/>
     <mergeCell ref="B72:I72"/>
-    <mergeCell ref="A54:A64"/>
     <mergeCell ref="A7:A32"/>
     <mergeCell ref="B43:I43"/>
     <mergeCell ref="B41:I41"/>
-    <mergeCell ref="B71:I71"/>
     <mergeCell ref="B49:I49"/>
     <mergeCell ref="B50:I50"/>
     <mergeCell ref="B40:I40"/>
@@ -4552,7 +4576,7 @@
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>AI pool (tainted)</t>
+          <t>AI GPU pool (tainted)</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
@@ -4859,7 +4883,7 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>AI pool: ticvai-ai, embeddings, reranker</t>
+          <t>AI GPU pool (the only AI pool): ticvai-ai, BGE-M3 and its reranker, Presidio and the Arabic NER</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">

</xml_diff>